<commit_message>
refactor: adaptado toda estrutura de driver para page objects de fato
</commit_message>
<xml_diff>
--- a/cypress/downloads/driver-01-07-2026.xlsx
+++ b/cypress/downloads/driver-01-07-2026.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="96">
   <si>
     <t>[ Name ]</t>
   </si>
@@ -63,36 +63,36 @@
     <t>[ Type ]</t>
   </si>
   <si>
+    <t>[ RG ]</t>
+  </si>
+  <si>
+    <t>[ CPF ]</t>
+  </si>
+  <si>
+    <t>[ E-mail ]</t>
+  </si>
+  <si>
+    <t>[ License Register ]</t>
+  </si>
+  <si>
+    <t>[ License Expedition ]</t>
+  </si>
+  <si>
+    <t>[ Birth date ]</t>
+  </si>
+  <si>
+    <t>[ Admission Date ]</t>
+  </si>
+  <si>
+    <t>[ Organizational Hierarchy ]</t>
+  </si>
+  <si>
     <t>[ License Category ]</t>
   </si>
   <si>
     <t>[ License Number ]</t>
   </si>
   <si>
-    <t>[ RG ]</t>
-  </si>
-  <si>
-    <t>[ CPF ]</t>
-  </si>
-  <si>
-    <t>[ E-mail ]</t>
-  </si>
-  <si>
-    <t>[ License Register ]</t>
-  </si>
-  <si>
-    <t>[ License Expedition ]</t>
-  </si>
-  <si>
-    <t>[ Birth date ]</t>
-  </si>
-  <si>
-    <t>[ Admission Date ]</t>
-  </si>
-  <si>
-    <t>[ Organizational Hierarchy ]</t>
-  </si>
-  <si>
     <t>[ RENACH ]</t>
   </si>
   <si>
@@ -162,24 +162,42 @@
     <t>Nordeste</t>
   </si>
   <si>
+    <t>Driver Modificado</t>
+  </si>
+  <si>
+    <t>200900</t>
+  </si>
+  <si>
+    <t>Caruaru</t>
+  </si>
+  <si>
+    <t>RFID</t>
+  </si>
+  <si>
+    <t>Inoperative</t>
+  </si>
+  <si>
+    <t>Seller</t>
+  </si>
+  <si>
+    <t>Nordeste / Pernambuco</t>
+  </si>
+  <si>
+    <t>123456789</t>
+  </si>
+  <si>
+    <t>Pernambuco</t>
+  </si>
+  <si>
     <t>Eduardo</t>
   </si>
   <si>
     <t>1998</t>
   </si>
   <si>
-    <t>Caruaru</t>
-  </si>
-  <si>
     <t>Permanent Contract</t>
   </si>
   <si>
-    <t>Nordeste / Pernambuco</t>
-  </si>
-  <si>
-    <t>Pernambuco</t>
-  </si>
-  <si>
     <t>Fabio</t>
   </si>
   <si>
@@ -204,6 +222,57 @@
     <t>20210417</t>
   </si>
   <si>
+    <t>Jose Driver da Silva</t>
+  </si>
+  <si>
+    <t>900101</t>
+  </si>
+  <si>
+    <t>Fortaleza</t>
+  </si>
+  <si>
+    <t>Introduce</t>
+  </si>
+  <si>
+    <t>GM-900101</t>
+  </si>
+  <si>
+    <t>01/01/2030</t>
+  </si>
+  <si>
+    <t>12345678900</t>
+  </si>
+  <si>
+    <t>12345678901</t>
+  </si>
+  <si>
+    <t>driver.complete@test.com</t>
+  </si>
+  <si>
+    <t>123456</t>
+  </si>
+  <si>
+    <t>01/01/2020</t>
+  </si>
+  <si>
+    <t>01/01/1990</t>
+  </si>
+  <si>
+    <t>01/07/2026</t>
+  </si>
+  <si>
+    <t>AB</t>
+  </si>
+  <si>
+    <t>987654</t>
+  </si>
+  <si>
+    <t>30100000</t>
+  </si>
+  <si>
+    <t>01/01/2015</t>
+  </si>
+  <si>
     <t>Leidson</t>
   </si>
   <si>
@@ -241,6 +310,15 @@
   </si>
   <si>
     <t>20210420</t>
+  </si>
+  <si>
+    <t>Zé Driver</t>
+  </si>
+  <si>
+    <t>900100</t>
+  </si>
+  <si>
+    <t>95297982</t>
   </si>
 </sst>
 </file>
@@ -612,7 +690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
@@ -762,13 +840,13 @@
         <v>34</v>
       </c>
       <c r="R2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="S2" t="s">
         <v>34</v>
       </c>
       <c r="T2" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="U2" t="s">
         <v>34</v>
@@ -818,10 +896,10 @@
         <v>45</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="F3" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="G3" t="s">
         <v>36</v>
@@ -830,10 +908,10 @@
         <v>34</v>
       </c>
       <c r="I3" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="J3" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="K3" t="s">
         <v>34</v>
@@ -857,13 +935,13 @@
         <v>34</v>
       </c>
       <c r="R3" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="S3" t="s">
         <v>34</v>
       </c>
       <c r="T3" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="U3" t="s">
         <v>34</v>
@@ -875,7 +953,7 @@
         <v>34</v>
       </c>
       <c r="X3" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="Y3" t="s">
         <v>34</v>
@@ -893,7 +971,7 @@
         <v>45</v>
       </c>
       <c r="AD3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="AE3" t="s">
         <v>42</v>
@@ -901,22 +979,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E4" t="s">
         <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G4" t="s">
         <v>36</v>
@@ -952,13 +1030,13 @@
         <v>34</v>
       </c>
       <c r="R4" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="S4" t="s">
         <v>34</v>
       </c>
       <c r="T4" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="U4" t="s">
         <v>34</v>
@@ -970,13 +1048,13 @@
         <v>34</v>
       </c>
       <c r="X4" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="Y4" t="s">
         <v>34</v>
       </c>
       <c r="Z4" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="AA4" t="s">
         <v>34</v>
@@ -985,10 +1063,10 @@
         <v>34</v>
       </c>
       <c r="AC4" t="s">
+        <v>45</v>
+      </c>
+      <c r="AD4" t="s">
         <v>51</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>41</v>
       </c>
       <c r="AE4" t="s">
         <v>42</v>
@@ -996,22 +1074,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" t="s">
         <v>54</v>
-      </c>
-      <c r="B5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" t="s">
-        <v>34</v>
-      </c>
-      <c r="F5" t="s">
-        <v>46</v>
       </c>
       <c r="G5" t="s">
         <v>36</v>
@@ -1047,13 +1125,13 @@
         <v>34</v>
       </c>
       <c r="R5" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="S5" t="s">
         <v>34</v>
       </c>
       <c r="T5" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="U5" t="s">
         <v>34</v>
@@ -1065,13 +1143,13 @@
         <v>34</v>
       </c>
       <c r="X5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="Y5" t="s">
         <v>34</v>
       </c>
       <c r="Z5" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="AA5" t="s">
         <v>34</v>
@@ -1080,7 +1158,7 @@
         <v>34</v>
       </c>
       <c r="AC5" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="AD5" t="s">
         <v>41</v>
@@ -1091,22 +1169,22 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="G6" t="s">
         <v>36</v>
@@ -1142,13 +1220,13 @@
         <v>34</v>
       </c>
       <c r="R6" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="S6" t="s">
         <v>34</v>
       </c>
       <c r="T6" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="U6" t="s">
         <v>34</v>
@@ -1160,7 +1238,7 @@
         <v>34</v>
       </c>
       <c r="X6" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="Y6" t="s">
         <v>34</v>
@@ -1175,10 +1253,10 @@
         <v>34</v>
       </c>
       <c r="AC6" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="AD6" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="AE6" t="s">
         <v>42</v>
@@ -1186,28 +1264,28 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D7" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G7" t="s">
         <v>36</v>
       </c>
       <c r="H7" t="s">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="I7" t="s">
         <v>37</v>
@@ -1216,75 +1294,75 @@
         <v>38</v>
       </c>
       <c r="K7" t="s">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="L7" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="M7" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="N7" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="O7" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="P7" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="Q7" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="R7" t="s">
         <v>34</v>
       </c>
       <c r="S7" t="s">
-        <v>34</v>
+        <v>76</v>
       </c>
       <c r="T7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="U7" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="V7" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="W7" t="s">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="X7" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="Y7" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="Z7" t="s">
         <v>40</v>
       </c>
       <c r="AA7" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="AB7" t="s">
         <v>34</v>
       </c>
       <c r="AC7" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="AD7" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="AE7" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="B8" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="C8" t="s">
         <v>45</v>
@@ -1293,7 +1371,7 @@
         <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>82</v>
       </c>
       <c r="F8" t="s">
         <v>35</v>
@@ -1332,13 +1410,13 @@
         <v>34</v>
       </c>
       <c r="R8" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="S8" t="s">
         <v>34</v>
       </c>
       <c r="T8" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="U8" t="s">
         <v>34</v>
@@ -1368,7 +1446,7 @@
         <v>45</v>
       </c>
       <c r="AD8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="AE8" t="s">
         <v>42</v>
@@ -1376,22 +1454,22 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="E9" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G9" t="s">
         <v>36</v>
@@ -1427,13 +1505,13 @@
         <v>34</v>
       </c>
       <c r="R9" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="S9" t="s">
         <v>34</v>
       </c>
       <c r="T9" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="U9" t="s">
         <v>34</v>
@@ -1445,7 +1523,7 @@
         <v>34</v>
       </c>
       <c r="X9" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="Y9" t="s">
         <v>34</v>
@@ -1460,18 +1538,303 @@
         <v>34</v>
       </c>
       <c r="AC9" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD9" t="s">
         <v>51</v>
-      </c>
-      <c r="AD9" t="s">
-        <v>41</v>
       </c>
       <c r="AE9" t="s">
         <v>42</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G10" t="s">
+        <v>36</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10" t="s">
+        <v>37</v>
+      </c>
+      <c r="J10" t="s">
+        <v>38</v>
+      </c>
+      <c r="K10" t="s">
+        <v>34</v>
+      </c>
+      <c r="L10" t="s">
+        <v>34</v>
+      </c>
+      <c r="M10" t="s">
+        <v>34</v>
+      </c>
+      <c r="N10" t="s">
+        <v>34</v>
+      </c>
+      <c r="O10" t="s">
+        <v>34</v>
+      </c>
+      <c r="P10" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>34</v>
+      </c>
+      <c r="R10" t="s">
+        <v>49</v>
+      </c>
+      <c r="S10" t="s">
+        <v>34</v>
+      </c>
+      <c r="T10" t="s">
+        <v>34</v>
+      </c>
+      <c r="U10" t="s">
+        <v>34</v>
+      </c>
+      <c r="V10" t="s">
+        <v>34</v>
+      </c>
+      <c r="W10" t="s">
+        <v>34</v>
+      </c>
+      <c r="X10" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>34</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>45</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E11" t="s">
+        <v>91</v>
+      </c>
+      <c r="F11" t="s">
+        <v>54</v>
+      </c>
+      <c r="G11" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" t="s">
+        <v>37</v>
+      </c>
+      <c r="J11" t="s">
+        <v>38</v>
+      </c>
+      <c r="K11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L11" t="s">
+        <v>34</v>
+      </c>
+      <c r="M11" t="s">
+        <v>34</v>
+      </c>
+      <c r="N11" t="s">
+        <v>34</v>
+      </c>
+      <c r="O11" t="s">
+        <v>34</v>
+      </c>
+      <c r="P11" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>34</v>
+      </c>
+      <c r="R11" t="s">
+        <v>39</v>
+      </c>
+      <c r="S11" t="s">
+        <v>34</v>
+      </c>
+      <c r="T11" t="s">
+        <v>34</v>
+      </c>
+      <c r="U11" t="s">
+        <v>34</v>
+      </c>
+      <c r="V11" t="s">
+        <v>34</v>
+      </c>
+      <c r="W11" t="s">
+        <v>34</v>
+      </c>
+      <c r="X11" t="s">
+        <v>92</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>34</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>57</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I12" t="s">
+        <v>37</v>
+      </c>
+      <c r="J12" t="s">
+        <v>38</v>
+      </c>
+      <c r="K12" t="s">
+        <v>34</v>
+      </c>
+      <c r="L12" t="s">
+        <v>34</v>
+      </c>
+      <c r="M12" t="s">
+        <v>34</v>
+      </c>
+      <c r="N12" t="s">
+        <v>34</v>
+      </c>
+      <c r="O12" t="s">
+        <v>34</v>
+      </c>
+      <c r="P12" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>34</v>
+      </c>
+      <c r="R12" t="s">
+        <v>34</v>
+      </c>
+      <c r="S12" t="s">
+        <v>34</v>
+      </c>
+      <c r="T12" t="s">
+        <v>34</v>
+      </c>
+      <c r="U12" t="s">
+        <v>34</v>
+      </c>
+      <c r="V12" t="s">
+        <v>34</v>
+      </c>
+      <c r="W12" t="s">
+        <v>34</v>
+      </c>
+      <c r="X12" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>34</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>34</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>